<commit_message>
articles on CC provided by Anna-Gwenn
</commit_message>
<xml_diff>
--- a/datasets/climate_change/climate_change_articles.xlsx
+++ b/datasets/climate_change/climate_change_articles.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacharles/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/annacharles/Desktop/PROCOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A12BD459-6545-4244-9C16-BB2DE605F069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E233AB9-3C4B-0A4D-97AC-AC9D94BCE4E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16380" xr2:uid="{F14E1FA3-A5AA-144B-9EA2-6E73000BB98F}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16380" xr2:uid="{07858322-9B94-EE4B-91EB-AA800797D44D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,44 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Climate Crazies Fail in Attempt to Vandalize Another Classic Work of Art 
+ Another of the world’s most recognized and most valuable pieces of art was the target of climate-change activists. Climate crazies tried — and failed — to glue themselves to Edvard Munch’s 1893 painting “The Scream” in Oslo on Friday.
+It was yet another example of climate change activists using priceless works of art to protest the use of fossil fuels, which climate zealots believe is leading to global warming. In October, climate activists attacked “Girl with a Pearl Earring” by Johannes Vermeer in The Hague. Climate hysterics were also responsible for an attack on Van Gogh’s “Sunflowers” and John Constable’s “The Hay Wain” in London over the summer.
+The new climate-related vandalism fad seems to have begun with an attack on Da Vinci’s “Mona Lisa” in which a climate fanatic feigned a disability in order to get close enough to smear a pastry on the painting.
+In addition, “Peach Trees in Blossom” by Van Gogh; “My Heart’s in the Highlands” by Horatio McCulloch; “Tomson’s Aeolian Harp” by J.M.W. Turner; “The Last Supper” by Giampietrino; “Sistine Madonna” by Raphael; and “Haystacks” by Monet have been targeted by climate hysterics since May.
+As of yet, none of the artwork has been damaged, due to being protected by glass.
+Video of Friday’s attack shows two young climate vandals attempting to glue themselves to the artwork. Police apprehended the hooligans, and reported there was some glue residue on the glass that protects the paintings.
+“I scream for people dying,” one of the activists shouted.
+“I scream when lawmakers ignore science,” the other shouted.
+The Norwegian climate activist group Stopp Oljeletinga, which translates to “Stop Oil Exploration,” claimed responsibility for the attack.
+The group demands that the Norwegian government declare “an immediate halt to all further exploration for oil on the Norwegian continental shelf,” and present “a concrete plan for fair adjustment for today’s oil workers.”
+A spokesperson for the group claimed that the vandalism was an attempt to “pressure lawmakers into stopping oil exploration.”
+“We are campaigning against ‘Scream’ because it is perhaps Norway’s most famous painting,” said Astrid Rem, a spokesperson for Stopp Oljeletinga. “There have been lots of similar actions around Europe. They have managed something that no other action has managed: achieve an extremely large amount of coverage and press.”
+But there’s good press and there’s bad press. These crazy antics are of the bad variety.
+Norway is one of the world’s top oil exporters and provides oil and natural gas to much of Europe, a continent in the midst of a serious energy crunch brought about partly by the war in Ukraine. Russia, the largest supplier of natural gas to Europe, has severely restricted supplies and has shut down the Nord Stream 2 pipeline, which it claims was sabotaged.
+Without much-needed Norwegian fossil fuels, Europe could be in for an extremely cold winter.
+The art world has acknowledged their concern over the new phenomenon:
+“In recent weeks, there have been several attacks on works of art in international museum collections. The activists responsible for them severely underestimate the fragility of these irreplaceable objects, which must be preserved as part of our world cultural heritage,” read a statement signed by approximately one hundred gallery directors and museums.
+These climate crazies are apparently willing to allow a continent to freeze this winter over their fears of an over-hyped “problem” peddled by globalists who flew more than 400 carbon-spewing private jets to COP27 in Egypt last week. If they truly believe the hype surrounding climate change, they’re targeting the wrong thing.</t>
+  </si>
+  <si>
+    <t>Climate Change Hoaxer Greta Thunberg Charged for Disobeying Law Enforcement in Sweden’s Climate Protest – May Face Up to Six Months in Prison 
+ Sweden says enough!
+Sweden’s Prosecution Authority is bringing charges against none other than their homegrown eco-hoaxer, Greta Thunberg, for disobeying law enforcement during a climate protest in June.
+The 20-year-old is facing potential fines or imprisonment of up to six months.
+The charges stem from her involvement in a protest that allegedly led to major traffic disruption in Malmö in June, authorities said.
+“The prosecutor has filed charges against a young woman who, on June 19 this year, participated in a climate demonstration which, according to the prosecution, caused disruption to traffic in Malmö,” the statement said. The woman “refused to obey the police command to leave the scene,” it added according to CNN.
+While the prosecution authority’s statement did not specifically name Thunberg, a spokesperson for the Swedish Prosecution Authority, Annika Collin, confirmed to CNN that the individual referred to in the charges is indeed Greta Thunberg.
+“The criminal classification is disobedience to law enforcement. According to the prosecutor, the act was committed with intent,” the prosecution authority’s statement added.
+Irma Kjellström, a spokesperson for Ta Tillbaka Framtiden, told CNN that Thunberg was among several young people who participated in blocking the oil tankers.
+Kjellström added, “After having blocked the industry which is burning our future, we have now been charged with crime. While charges are being brought against us, the real crime continues inside the gates that we blocked.”
+Recently, Greta Thunberg was back in the news after her prediction that the world would end in 2023 was a conspiracy.
+On June 21, 2018, she made a bold claim on Twitter, stating that humanity had a narrow five-year window to stop the use of fossil fuels or face inevitable extinction.
+“A top climate scientist is warning that climate change will wipe out all of humanity unless we stop using fossil fuels over the next five years.”
+Thunberg shared a now-deleted Grit Post article by Scott Alden citing a prediction from James Anderson, a professor of atmospheric chemistry at Harvard University, titled, “Top Climate Scientist: Humans Will Go Extinct if We Don’t Fix Climate Change by 2023.”</t>
+  </si>
   <si>
     <t>Text-ID</t>
   </si>
@@ -46,56 +83,7 @@
     <t>CC_001</t>
   </si>
   <si>
-    <t>Kenya has revealed why it is pushing to ensure that the global financial architecture towards climate change undergoes urgent reforms.Prime Cabinet Secretary Musalia Mudavadi said developing countries such as Kenya have a challenge balancing development and addressing the impacts of climate change.“We already dealing with a lot of public debt through expensive funding. So if you can re-engineer and then have it concession and when I say concessional, that means borrowing at even one per cent or less, and having a longer period of repayment, maybe even 30 to 40 years, so that countries can actually push the Climate Action Agenda without devastating the overall fabric in their countries. So this is going to be very, very important,” Mudavadi said.Mudavadi is leading Kenya’s delegation to the ongoing climate talks in Azerbaijan. Environment CS Aden Duale and Environment PS Festus Ng’eno are also taking part in the talks.World leaders and negotiators are in Baku, Azerbaijan, for the United Nations Climate Change Conference, known as the 29th Conference of Parties (COP29).Kenya is among countries pushing to have more resources to address the impacts of climate change.African countries want $1.3 trillion annually to meet the realities of climate impacts.Duale echoed Musalia’s sentiments adding that Kenya needs grants to tackle climate change and not expensive loans. He said Kenya has put in place policies and regulations especially those touching on carbon credits.He said communities are set to benefit.“It's in that regulation, it's in law that 40 per cent of any carbon projects will be done in any place in our country. 40 per cent will go to the local community in terms of education, healthcare, making sure what is available,” Duale said.UN Secretary-General António Guterres urged providers of bilateral and multilateral funds to redouble their efforts, to help cover investment gaps.“We need to encourage private finance, particularly through public-private partnerships. And we need to simplify access to early warning system finance. And to massively increase the sums available. Increasing the lending capacity of the Multilateral Development Banks is key. The Pact for the Future agreed in September made important strides forward,” he said."</t>
-  </si>
-  <si>
     <t>CC_002</t>
-  </si>
-  <si>
-    <t>Hello friends, how are you? How are we?Last week a student in the class I am teaching at Hamline University shared this website that tracks how the worldâ€s countriesâ€ actions are on track for meeting the Paris Agreement goal to keep temperatures within a 1.5â„ƒ increase. It assigns each country, based on its actions, to one of 5 categories: critically insufficient, highly insufficient, insufficient, almost sufficient, and 1.5â„ƒ compatible. I shared it with my team here at Climate Generation via Slack. On Thursday, I walked into our shared room and found a coworker, seated quietly with her hand across her heart, breathing slowly and intentionally, with this same website open on her laptop.You see,there are zero nations whose actions are ambitious enough to limit warming . The UNFCCC Conference of the Parties 29 started this week in Baju, Azerbaijan. I hope you are signed up to receive the Digest and follow our amazing delegates. For the third year in a row, a petrostate with human rights issues is hosting this critical conference. My expectations are low for this diplomatic space where there is no accountability and everyone seems to show up for their own nationâ€s interests instead of what is best for all of us and the planet. The United States just elected a convicted felon, sex offender, and climate change denier to the presidency. It is highly likely that federal agencies and programs that have been providing climate literacy resources, environmental justice action and climate adaptation resources will go dark. And, while I know what this means for the planet and our collective future, I am more sure than ever that the work we do here at Climate Generation â€” igniting and sustaining the ability of youth, educators and community to fight the systems perpetuating the climate crisis â€” is more important than ever. The only way we push back against mis- and disinformation is to educate, organize and build intergenerational power for climate justice. The only way we are prepared to transition to a viable future is through climate change literacy and climate justice education.We are ready for the challenge ahead. Will you join us?"</t>
-  </si>
-  <si>
-    <t>CC_003</t>
-  </si>
-  <si>
-    <t>international cocoa prices have experienced a historic price surge , rising by over 300% in the space of 12 months from £2,166 per tonne of cocoa in April 2023 to £9,980 by April 2024. Prices have fallen since then, and are currently hovering around the £6,400 mark at the time of writing.This rally, which is the highest on record for cocoa, was driven by poor harvests in the Ivory Coast and Ghana. Powerful El Niño weather events , coupled with years of underinvestment that left Ghana’s cocoa trees vulnerable to diseases, have decimated yields.In February 2024 Ghana’s cocoa board, Cocobod, revised its cocoa crop forecast down 40% from its initial target of 820,000 metric tonnes for the 2023-24 season. Ghana and the Ivory Coast account for nearly 60% of global cocoa production, so markets reacted to the news swiftly.We are researchers of the global cocoa trade, and one of us is particularly familiar with the mechanics of Ghana’s cocoa sector. Fuad is currently the head of the Ghana Cocoa Marketing Company UK, which facilitates trade transactions between the Cocoa Marketing Company Ghana (CMC) – a subsidiary of Cocobod and the monopoly seller of Ghanaian cocoa beans – and its clients across the world.The tripling of cocoa prices in London, which serve as the benchmark for west African cocoa, should have been a blessing for Ghana’s economy and its cocoa farmers, many of whom have long struggled with low incomes. However, the prices farmers are paid for their cocoa (farmgate prices) remained well below international market prices despite the extraordinary surge.Cocobod increased farmgate prices by 58% in April, followed by another 45% hike at the start of the 2024-25 season in September. This latter move increased the price farmers are paid per tonne of cocoa from 33,120 Ghanaian cedis (£1,599) to 48,000 Ghanaian cedis (£2,304).A further 3.3% price increase was announced by Ghana’s president, Nana Akufo-Addo, during the celebration of Ghana’s National Farmer’s Day on November 8 in a bid to motivate cocoa farmers.These price hikes are significant, but they have not kept pace with the movement in the global benchmark. This has led to a growing gap between farmgate prices in Ghana and the Ivory Coast, and the international market.In our recent working paper , we show that the limited pass-through of global prices to farmers in Ghana was primarily due to the combined effect of a longstanding forward sales strategy and a financing structure that relies on a loan sourced from a group of international banks (a syndicated loan).For decades, the CMC has used forward sales to hedge against downward trending prices. This involves selling up to 70% of the anticipated cocoa crop between nine and 12 months ahead of harvest to international traders and local processors at prices tied to the global benchmark.The average price secured through these contracts is then used to set farmgate prices before the start of each cocoa season. This system protects farmers from price drops in a declining market, but it does not allow them to benefit if the spot price at harvest is above the forward price that is achieved by the CMC.With a near-tripling of cocoa prices in only 12 months, the average forward prices secured by the CMC were significantly lower than the levels achieved in international spot markets. This limited the potential for a substantial increase in farmgate prices.Besides price risk management, the forward sales fulfil another role. For over 31 years, Cocobod has relied on a syndicated loan to finance the purchase of cocoa beans from farmers, as well as farming inputs such as fertilisers and jute bags. The forward contracts are used as collateral against which the loan is drawn.Cocobod has raised nearly US$28 billion (£21.6 billion) through the loan since its inception. Given the size of the cocoa sector in the overall economy – cocoa has ranked consistently among Ghana’s top four exports over the past three decades – the loan’s importance goes beyond the cocoa trade.The loan has provided the Ghanaian central bank with the ability to borrow hard currency at affordable interest rates. Hard currency is needed to pay for imports and to stock up on foreign exchange reserves. This is particularly needed now as Ghana’s debt crisis has made other means of external borrowing more challenging since 2021.Because of the need for collateral to secure the loan, forward contracts must be signed and prices locked in before the season starts. This limits the volume of cocoa that can be sod at a more favourable spot price when market conditions improve.A downward trending cocoa price over the longer term remains a concern. But extreme weather caused by climate change, and the resulting increased market volatility, have put into question the sustainability of both the forward sales system and the loan.So, in August 2024 the chief executive of Cocobod, Joseph Boahen Aidoo, announced that Ghana would not raise a loan for the 2024-25 season. The decision to end three decades of dependency on this financing model was made in light of significantly higher interest rates, which has made offshore borrowing much less attractive.Cocobod’s new financing model requires licensed buying companies (LBCs), which are responsible for purchasing cocoa beans from farmers at the price set by Cocobod, to secure funding independently. Previously, they received centralised funding from Cocobod through the loan.Under this new system, LBCs primarily source funding from international cocoa traders and, to a lesser extent, domestic banks. The LBCs buy cocoa from farmers with the secured funding and deliver it to the CMC. They are then reimbursed for the amount they paid farmers for the beans plus an agreed margin for their service by Cocobod.However, the need for LBCs to secure their own financing within a short planning window poses challenges for some in the 2024-25 season, particularly as local firms face hurdles in accessing affordable domestic credit. In an effort to ensure sufficient volumes, many international traders have established sourcing partnerships with local buyers. But some local buyers argue that this could further consolidate power among multinational firms because the buyers would essentially become beholden to them.Ghana’s 31-year reliance on the cocoa-backed loan has constrained its ability to fully capitalise on price rallies. The shift to a new financing model grants the CMC flexibility to time its cocoa sales, utilising both forward and spot contracts. It also has the potential to improve cash liquidity for Ghana’s cocoa buying companies. With proper execution and commitment by Cocobod to ensure timely reimbursement, this approach could reshape Ghana’s cocoa industry and significantly improve the livelihoods of nearly 1 million cocoa farming families."</t>
-  </si>
-  <si>
-    <t>CC_004</t>
-  </si>
-  <si>
-    <t>WASHINGTON, Nov 19 –– The world’s richest man, Elon Musk, has been an ever-present sidekick for President-elect Donald Trump since the US election at the start of the month.“I can’t get him out of here,” Trump joked about Musk at his Mar-a-Lago resort in Florida last Thursday. “I like having him here as well. He’s done a fantastic job, an incredible mind.”But can the bromance between the world’s wealthiest man and the soon-to-be US president survive some major policy differences and their own combustible personalities?AFP looks at six possible areas of friction:Who’s the boss?Musk is famed for his manic working habits and self-described “hardcore” style, running his companies as personal fiefdoms in which his authority is rarely challenged.From factory production lines to the boardroom, he is used to getting his way with an abrasive style that sees him fire people on the spot and sometimes insult their intelligence in public. Trump, also a tycoon fond of firing and humiliating people publicly, demands total loyalty and has chafed against sharing the limelight with others in the past.He also likes to play his advisors and cabinet members against each other, former aides say.Musk reportedly had a first public row with Trump transition official Boris Epshteyn last week, according to the Axios news site.And he openly endorsed brokerage billionaire Howard Lutnick for US Treasury secretary on Saturday, setting up an early test of his influence.Climate changeMusk invested in Tesla in 2004 partly out of concern about global warming.In 2017, he resigned from Trump’s business advisory councils to protest the then-president’s decision to pull the United States out of the Paris climate change accord.“Climate change is real. Leaving Paris is not good for America or the world,” Musk wrote on Twitter at the time.Trump, who has called climate change a “hoax,” is widely expected to abandon US commitments again after President Joe Biden re-joined the Paris Accord in 2020.Musk has shifted his views recently, telling Trump during a live conversation on X in August that “if 50-100 years from now we’re mostly sustainable I think that will probably be OK.” The world’s top climate scientific body, the UN’s IPCC, says average global temperatures are on track to reach 1.5C above pre-industrial times in the early 2030s, a key level with major consequences for ecosystems.Energy transitionMusk has bet big on the energy transition, making his fortune from Tesla electric cars, but also developing domestic battery technology and solar-powered roof tiles.Trump ran pledging to “drill, baby, drill” and is expected to approve new fossil fuel infrastructure and permits, even opening up protected federal land to oil and gas companies.Musk used to deride the “mine-and-burn hydrocarbon economy” thatTrump openly champions.The president-elect has nominated a fracking magnate as his energy secretary. Chris Wright publicly dismissed climate change and the energy transition last year.ChinaTrump’s aggressive stance on China and the risk of a trade war between the world’s two biggest economies could be another major thorn in the relationship between the billionaires.China is a major market for Tesla, where the company has one of its so-called “Gigafactories” and is trying to compete with fast-growing home-grown manufacturers.Musk never says a negative word about the ruling Communist Party, putting him at odds with the China hawks like US Senator Marco Rubio who have been tapped to join Trump’s cabinet.‘DOGE’ on a leashAn unsparing cost-cutter in his own companies, Musk has been tasked by Trump with leading the “Department of Government Efficiency (DOGE),” which will take an ax to government spending.Plans to gut programs will almost certainly, however, face severe political pushback, even from Republicans.As mid-term elections approach, whether it’s rescuing Medicaid checks for the poor or handing out defense contracts to benefactors, Trump’s political priorities could waver from Musk’s.Big techMusk’s complicated relationships and personal rivalries with Silicon Valley’s biggest tech companies go back decades, and he is expected to face myriad conflicts of interest  as part of the administration.Would Musk, who owns his own AI company, sit by quietly if Trump champions OpenAI, the Microsoft-backed startup that Musk played a key role in starting a decade ago? If Amazon founder Jeff Bezos gets Trump’s ear, would Musk tolerate that a rival to SpaceX got closer to the White House inner sanctum? –– Reuters"</t>
-  </si>
-  <si>
-    <t>CC_005</t>
-  </si>
-  <si>
-    <t>Limos4 commits to reaching net-zero carbon emissions by 2040 or sooner. BUCHS, SWITZERLAND, November 19, 2024 /EINPresswire.com/ -- Today, Limos4 announced its commitment to The Climate Pledge. Limos4, a global provider of premium chauffeured ground transportation, is dedicated to integrating sustainability into its operations and services by enhancing environmental responsibility across all business aspects. As part of its -commitment to the environment, Limos4 actively pursues initiatives to reduce its carbon footprint while upholding its uncompromising standards of service excellence, ensuring that sustainability and quality remain integral to its operations.Co-founded by Amazon and Global Optimism in 2019, The Climate Pledge is a commitment by companies to reach net-zero carbon emissions by 2040 — a decade ahead of the Paris Agreement’s goal of 2050. Signatories to The Climate Pledge agree to:Measure and report greenhouse gas emissions on a regular basis.Implement decarbonization strategies in line with the Paris Agreement through real business changes and innovations, including efficiency improvements, renewable energy, materials reductions, and other carbon emission elimination strategies.Neutralize any remaining emissions with additional, quantifiable, real, permanent, and socially beneficial offsets to achieve net-zero annual carbon emissions by 2040 — a decade ahead of the Paris Agreement’s goal of 2050.Limos4’s Sustainability Initiatives:As a company deeply committed to sustainability, Limos4 is not only enhancing but actively expanding its initiatives, with a focused approach on reducing emissions and improving energy efficiency throughout its operations. Electric Vehicle Integration: Limos4 is introducing electric vehicles across its global fleet, significantly reducing emissions and moving toward zero emission transportation.Sustainability Dashboard/Reports: Clients have access to real-time CO2 tracking, offering transparency into their carbon footprint and enabling informed travel decisions.Sustainable Partnerships: Limos4 selects partners based on their sustainability credentials, ensuring eco-friendly practices across its supply chain.AI-Driven Efficiency: Limos4 employs AI technology to optimize routing and scheduling, reducing fuel consumption and operational waste, while also improving client interaction efficiency.Limos4 Executive Quote:“We are running out of time to avoid the worst impacts of climate change, and as a global company, we recognize our responsibility to lead by example in the transportation industry. Achieving net-zero by 2040 is a crucial step for our planet, and Limos4 is proud to join The Climate Pledge. Together, with other signatories, we will create a more sustainable future through innovation, collaboration, and collective action.” said Dr. Vojkan Tasic, CEO of Limos4.About Limos4Limos4 sets the gold standard in global chauffeured ground transportation, offering tailored solutions for corporate, executive and event transportation needs in over 200 cities worldwide. Driven by innovation and sustainability, Limos4 combines cutting-edge technology with a rigorous five-step quality control process to deliver a consistently seamless experience. Trusted by Fortune 500 companies, prominent institutions, and high-end leisure travelers, Limos4 is known for its strong commitment to safety, efficiency, and client satisfaction. Discover more at www.limos4.com.About The Climate Pledge In 2019, Amazon and Global Optimism co-founded The Climate Pledge, a commitment to reach the Paris Agreement 10 years early and be net-zero carbon by 2040. Over 525 organizations have now signed The Climate Pledge, sending an important signal that there will be rapid growth in demand for products and services that help reduce carbon emissions."</t>
-  </si>
-  <si>
-    <t>CC_006</t>
-  </si>
-  <si>
-    <t>From day one of his Administration, President Biden pledged to restore U.S. leadership and strengthen our partnerships to make America more secure and prosperous. Taking office amid a devastating pandemic that had upended the global economy, President Biden recognized that we needed to work with partners to tackle big cross-border challenges.  President Biden's leadership at the G20 has demonstrated the dividends that U.S. engagement yields for America and the world. Through the G20, the Biden-Harris Administration has delivered a landmark agreement to stop the race to the bottom in corporate taxation; launched a new fund to address pandemic threats; and helped unlock hundreds of billions of dollars of resources at the international financial institutions to advance development progress and tackle global challenges.At the Rio Summit, President Biden continued this legacy of leadership by rallying his fellow leaders to unlock space for developing countries to invest in their futures, accelerate the global clean energy transition, tackle global health threats, and champion an inclusive digital transformation. He also built on the United States' longstanding leadership on food security by joining the Global Alliance Against Hunger and Poverty.President Biden continued his push for peace and stability around the world. He condemned Russia's brutal invasion of Ukraine - which has exacerbated the crises facing developing countries - and affirmed the United States' strong support for Ukraine's sovereignty and territorial integrity and called on his fellow leaders to do the same. President Biden also affirmed Israel's right to defend itself while emphasizing that how it defends itself - even as Hamas cruelly hides among civilians - matters. He highlighted U.S. humanitarian aid to Gaza and made clear that the United States is pushing for a ceasefire deal that ensures Israel's security, brings the hostages home, and ends the suffering of Palestinians in Gaza. President Biden asked his fellow leaders to increase pressure on Hamas to stop refusing this deal.Driving sustainable growth and development in developing countriesPresident Biden has built his economic agenda around the United States investing at home and unlocking additional resources to support investments in developing countries around the world.Championing concessional finance from the World Bank for the poorest countries. President Biden announced the U.S. intent for a substantial increase in the U.S. contribution to the International Development Association (IDA), the arm of the World Bank that supports the poorest and most vulnerable countries. The Biden Administration intends to pledge $4 billion over three years to the ongoing IDA replenishment, subject to Congressional approval. A better and bigger IDA is critical to unlocking space for developing countries to invest in their futures. President Biden has heard loud and clear the calls from developing countries for more concessional financing and a strong IDA replenishment in December. This pledge will sustain U.S. leadership as the largest historical donor to IDA and joins other countries that are stepping up to support IDA recipients with critical, sustainable investments in their development. At the Rio Summit, President Biden called on existing donors to follow the U.S. example by increasing support and on new donors to start contributingEquipping the multilateral development banks (MDBs) to address global challenges. The Biden-Harris Administration has spearheaded a broad coalition to equip the MDBs to better address global challenges like climate change, pandemics, and fragility and conflict. Over the last two years, this leadership has led to enormous strides in reforming the MDBs' visions, incentives, and operations to make them more efficient and responsive to countries' development needs. Reforms already identified could boost lending capacity by up to nearly $360 billion over the next decade, giving the MDBs the resources they need to tackle global challenges with greater speed and scale. At the Rio Summit, President Biden reiterated his request for Congress to approve funding to boost World Bank lending capacity by $36 billion, recognized the G20 members that have made their own contributions to this U.S.-led effort, and called on fellow leaders to match this with their own contributions.Unlocking space for developing countries to invest in sustainable growth and development. High debt service burdens are preventing developing countries from making critical investments in their futures - many low-income countries spend more servicing their debt than on health, education, and social programs combined. Building on the Nairobi-Washington Vision that he launched with President Ruto of Kenya in May 2024, President Biden called on the G20 to provide a pathway for sustainable growth for these countries that would bring together the international community to provide stepped-up support for countries facing constraints from debt servicing burdens, but whose debts are sustainable. Under this plan, the IMF and MDBs would deliver enhanced support packages that incorporate ambitious reform and investment agendas; bilateral creditors would provide net positive financial flows to end free-riding; and MDBs and G20 countries would deploy their tools to unlock private financing. As part of this plan, the U.S. government is employing its multilateral and bilateral tools to step up financing for vulnerable countries. This includes finalizing the U.S. contribution of $21 billion to the IMF's Poverty Reduction and Growth Trust.Calling for faster debt relief for countries with unsustainable burdens. President Biden pushed for making the debt restructuring process faster and more predictable to reduce the hardship on the people of indebted countries. President Biden called on G20 countries to swiftly provide debt relief to countries who need it and advocated for accelerating the restructuring process, including by improving the G20 Common Framework.Furthering the global clean energy transitionAfter a historic visit to the Amazon that highlighted his legacy of spearheading the most significant domestic climate and conservation action in history and leading global efforts to tackle the climate crisis through a historic pledge to increase U.S. international climate finance to over $11 billion a year by 2024, President Biden rallied G20 leaders in Rio to raise their climate ambition and develop innovative solutions to support the clean energy transition.Launching the Brazil-U.S. Partnership for the Energy Transition. Presidents Biden and Lula announced a new partnership to elevate ongoing bilateral efforts in clean energy production, clean energy supply chain development, and green industrialization. This partnership builds on longstanding efforts under the U.S.-Brazil Energy Forum and the Strategic Minerals Dialogue. This partnership will also help mobilize private sector investment in the energy transition through engagement under the Clean Energy Industry Dialogue and the recently signed cooperation framework agreement between the U.S. International Development Finance Corporation (DFC) and BNDES, the Brazilian Development Bank.Globalizing the U.S. clean energy industrial strategy. The United States has demonstrated that investing in the energy transition is a once-in-a-generation opportunity to unlock clean growth, good jobs, high-standard investment, and energy security. This vision is reflected in a number of bilateral clean energy industrial partnerships President Biden has established, including the new Brazil-U.S. Partnership for the Energy Transition, Roadmap For U.S.-India Initiative to Build Safe and Secure Global Clean Energy Supply Chains, and U.S.-Kenya Climate and Clean Energy Industrial Partnership. These efforts are further cemented in the multilateral Clean Energy Finance Mission Statement released on the margins of the G20 under the leadership of the United Kingdom and Brazil to mobilize finance in emerging markets and developing economies (EMDEs) for green industrialization and building resilient and diverse clean energy supply chains.U.S. leadership in financing the global clean energy transition. Alongside the Clean Energy Finance Mission Statement, the United States announced a major $325 million contribution to the Clean Technology Fund, a highly concessional fund designed to support the scaling and diversification of clean energy supply chains in eligible EMDEs. The United States has also separately extended $2 billion in shareholder guarantees through the World Bank to catalyze India's and Indonesia's investments in the clean energy economy.Reforming the multilateral climate funds. After leading the effort to equip the MDBs to better address global challenges like climate change, the United States is working with others to reform the vertical climate and environmental funds as the next frontier in the evolution of the international financial architecture. Building on an independent review of the funds launched by the G20 this year, G20 leaders encouraged the funds to work together to unlock their full potential and improve access, including through enhanced cooperation with the MDBs. This call to action can pave the way for the funds to deliver finance at the speed and scale the climate crisis demands.Strengthening the global health architecture When he came into office, President Biden prioritized ending the COVID-19 pandemic and preparing for future pandemics. At the Rio Summit, President Biden built on this legacy to continue tackling the threat of pandemics and delivering for global health.Delivering for the Pandemic Fund. President Biden led the G20 to establish the Pandemic Fund in 2022 to help developing countries build capacity to prepare, prevent, and respond to the next pandemic. In its first two years, the Pandemic Fund has awarded $885 million in grants across 75 countries, including nearly $129 million for countries affected by the mpox public health emergency, and mobilized an additional $6 billion in co-financing and co-investment for project implementation, delivering support that is making America - and the world - safer from the next pandemic threat. The United States is championing an ambitious $2 billion replenishment of the Pandemic Fund and leading the way by pledging up to $667 million by 2026, subject to Congressional approval. At the Rio Summit, the United States led a G20 call for new and increased contributions to reach the funding goal.Responding to the threat of mpox. The United States galvanized the G20 to commit political and financial support to the mpox response and support the World Health Organization (WHO) and the World Bank in creating a global mpox response financing tracker to identify and address gaps. The financing tracker, which will be launched soon, shows that countries have stepped up quickly, providing 90 percent of the resources needed to respond, including more than $540 million from the United States. The United States has also pledged to provide more than one million mpox vaccine doses to the response. Nearly 400,000 doses have already been allocated through WHO and Africa CDC's Access and Allocation mechanism; the remaining doses will be allocated as guided by country requirements.Restoring immunization services to better than pre-pandemic levels. In June, the United States pledged at least $1.58 billion over the next five years to Gavi, the Vaccine Alliance, the first-ever five-year pledge and the largest-ever U.S. pledge. In Rio, President Biden called on other countries to come forward with their own ambitious pledges in support of Gavi's goal of vaccinating an additional 500 million children and saving at least 8 million lives. In September 2024, DFC expanded its donor liquidity partnership with Gavi, building on support put in place during COVID-19. The $1 billion Rapid Financing Facility will allow Gavi to access funds from donors making new pledges for pandemic response or routine immunization much faster.Ending HIV/AIDS, tuberculosis, and malaria as public health threats by 2030. The Biden-Harris Administration has invested more than $26 billion in the HIV/AIDS response. Through the President's Emergency Plan for AIDS Relief (PEPFAR), the Administration has supported more than 20 million people on lifesaving treatment and reached millions more with effective HIV prevention programs. In 2022, President Biden led the largest ever replenishment for the Global Fund to Fight AIDS, Tuberculosis, and Malaria (Global Fund), raising more than $15.7 billion in donor pledges, including a U.S. pledge of $6 billion over three years. President Biden also sustained robust bilateral funding for the President's Malaria Initiative, which provided more than $3 billion for malaria to support 30 countries who together account for around 90 percent of all malaria cases and deaths globally.Addressing the environmental determinants of health. President Biden led G20 members to emphasize the importance of addressing One Health (human-animal-plant-environment) challenges such as antimicrobial resistance (AMR) and climate change. On AMR, the Administration has invested $1 billion to prevent infections and detect and respond to AMR and has finalized policies aimed at preventing the rise of AMR due to crop pesticide use. On climate and health, the Administration has included health as one of four key sectors for its PREPARE action plan. The over $3 billion invested through PREPARE supports resilient health systems while also supporting key life support systems such as food, water, and infrastructure. At home, the Administration has launched a first-of-its kind National Heat Strategy and secured the commitment of more than 960 health care companies to address their emissions and climate resilience.Leading the fight against poverty and hungerPresident Biden built on the United States' longstanding leadership on global food security.Accelerating progress on global food security. In the face of a protracted global food security crisis, the Biden-Harris Administration has led the fight against global hunger. Since 2021, the United States has committed more than $20 billion in funding in more than 47 countries to support emergency interventions and build more resilient and sustainable food systems to mitigate against future global food shocks. In 2022, the Biden-Harris Administration rallied more than 100 countries to endorse the UN Roadmap for Global Food Security, affirming the importance of tackling global food insecurity as an economic and national security imperative.Launching G20 action on hunger and poverty. At the Rio Summit, President Biden joined G20 leaders to launch the Global Alliance Against Hunger and Poverty to provide sustained political momentum and facilitate better alignment of financial resources and knowledge-sharing in support of efforts with a proven track record of impact in accelerating the eradication of poverty. As a member of the Alliance, the United States highlighted existing U.S.-led efforts to reduce malnutrition, increase women's access to land tenure, and promote private sector investments in improved seed varieties globally. President Biden also highlighted a number of domestic efforts to lift millions of people in the United States out of poverty through the Social Security program, nutrition assistance, refundable tax credits, and benefits for disabled Americans.Combatting corruption to drive sustainable and equitable development. Recognizing that corruption and weak governance impede the Sustainable Development Goals, the United States is working with partners to press for stronger action to prevent and counter corruption, including better enforcement by all G20 countries of foreign bribery laws and ensuring transparent, inclusive, and accountable public institutions.Empowering workersIn September 2023, Presidents Biden and Lula launched the Partnership for Workers' Rights, the first joint U.S.-Brazil initiative to advance the rights of working people around the world. The Partnership has tangibly improved the lives of workers through new initiatives and over $20 million of programming supported by the United States that:Facilitated collaboration to prevent heat-related illnesses and promoted the use of mobile apps and other tools to help workers know when they are at risk of heat-related illnesses.Advanced collaborative efforts with businesses, governments, and unions to tackle the root causes of forced labor and promote forced labor remediation, including in the cattle, coffee, gold mining, charcoal production, and other industries and supply chains.Supported efforts to strengthen worker engagement in climate policy and promoted unionization and collective bargaining in the manufacturing and agriculture sectors.Supporting an inclusive and equitable digital future for allRecognizing the potential of the digital transformation to empower people globally, President Biden advocated for an inclusive and equitable digital future for all in Rio.Leveraging artificial intelligence (AI) for sustainable development and worker empowerment. President Biden joined other G20 Leaders in advocating to leverage the potential of AI to help solve global challenges, enable worker well-being, and ensure AI technologies are developed and used responsibly. The United States has demonstrated its commitment to achieving this goal by delivering on President Biden's Executive Order on AI, particularly the AI in Global Development Playbook and the Global AI Research Agenda.Making progress on universal and meaningful connectivity. President Biden proudly joined other G20 leaders in recognizing universal and meaningful connectivity as key to achieving digital inclusion. To help achieve this, DFC has approved a combined $630 million in financing for the Brazilian digital infrastructure company V.tal Rede Neutra De Telecomunicacoes S.A. (V.tal) to support the expansion of its fiber optic network across Brazil. DFC's financing will enable more than 1 million homes and 4,000 schools to be connected to the Internet by 2027.Investing through the Women in the Digital Economy Initiative. G20 leaders reaffirmed the historic commitment from the 2023 G20 Leaders' Summit to halve the digital gender gap by 2030. In furtherance of this commitment, the United States announced the first round of global funding awards through the Women in the Digital Economy Initiative's aligned fund. Ten organizations, spanning eight countries across East Africa, West Africa, South Asia, and Latin America, have been selected for their innovative solutions and impact in tackling the gender digital divide. These organizations will address barriers to equitable digital inclusion, such as access to affordable devices and online experiences; availability of relevant products and tools; digital literacy and skills; safety and security; and data and insights."</t>
-  </si>
-  <si>
-    <t>CC_007</t>
-  </si>
-  <si>
-    <t>New Delhi: As India looks to achieve energy security amid growing demand, Periasamy Kumaran, special secretary at the external affairs ministry said India should secure supply chains for nuclear fuel and develop indigenous technologies to increase the share of nuclear power in its energy mix.Speaking at the CII Energy Security Conference in New Delhi on Tuesday, Kumaran noted that India’s energy transition has drawn the country into global supply chains of solar modules, wind-turbines, critical minerals and semiconductors, and that control over these resources could cause geopolitical tensions and give rise to new coalitions.The Indian government is looking to increase India’s nuclear power capacity from 7 GW at present to 22 GW by 2032 and has identified 18 potential sites to set up nuclear power plants. It hopes nuclear power will play a key role in helping the country achieve its target of 500 GW of non-fossil-fuel energy by 2030.Coal is king“Coal is the backbone of our power generation, accounting for 17% of energy production, and is seen as an affordable and viable source of energy. With substantial coal reserves, India uses coal to buffer its energy security, especially during periods of high demand and shortages,” Kumaran said.Pallavi Jain Govil, director general of the Directorate General of Hydrocarbons (DGH) said at the conference that oil and gas exploration is set to begin in the Andaman Basin, with hopes of a major discovery. “We are hoping that the exploration in the Andaman basin will turn out to be the new Mumbai High for us,” she said. Govil underscored the importance of high-quality geological data to attract investments, and announced efforts to move India’s National Data Repository (NDR) to the cloud to improve data accessibility and sharing. Virendra Gupta, co-chairman of the CII Core Group on Energy Security and president of the Indian Council for International Cooperation, said India has been diversifying its sources of oil beyond West Asia to other regions, including Africa. “At one point, acquiring energy assets abroad was equated with energy security. But that may not be the case, for instance, in a war. Even if you own an energy asset, shipping it to India can be difficult. At the most, it insulates against price shocks,” he said."</t>
-  </si>
-  <si>
-    <t>CC_008</t>
-  </si>
-  <si>
-    <t>Leaders of the Group of 20 major economies meet on Tuesday to discuss sustainable development and the transition to cleaner energy, as they aim to increase the odds of a successful deal to address global warming at U.N. climate talks in Azerbaijan.The host of the COP29 climate summit a day earlier had made a plea for G20 countries to send a positive signal on the need to tackle climate change and provide clear mandates to help save talks that had bogged down in Baku, Azerbaijan.With the world on track for its warmest year on record, leaders are trying to shore up a global response to climate change before Donald Trump retakes the U.S. presidency in January. He is reportedly preparing to roll back U.S. policy on global warming and exit the landmark Paris Agreement.The G20 leaders gathering for a summit in Rio de Janeiro, Brazil, called in a joint statement on Monday for "rapidly and substantially increasing climate finance from billions to trillions from all sources to respond to global warming.They also urged COP29 negotiators to reach a deal on a new financial goal for how much money rich nations must provide to poorer developing nations in climate finance, the main sticking point in the climate talks.G20 Leaders have sent a clear message to their negotiators at COP29: do not leave Baku without a successful new finance goal. This is in every country's clear interests, U.N. climate chief Simon Stiell said in a statement.Climate negotiators aim to produce a full draft of a deal for the financial goal by Wednesday evening, said the summit's lead negotiator Yalchin Rafiyev of Azerbaijan.We have stepped up the pace," Rafiyev said. "The outcome will only be as good as parties' commitment to help us build solutions.VAGUENESS While negotiations, slated to conclude on Friday, have yet to coalesce around a specific number, economists suggest the goal should be at least $1 trillion annually.The G20 statement said nations need to break the impasse on finance, but they did not give clear guidance on a solution. Some activists called the G20 statement weak on climate finance."This vagueness of the G20 declaration risks undermining trust in the negotiations, as the G20's influence is crucial for bridging the divides between developed and developing nations,said long-time activist Oscar Soria, head of The Common Initiative, an environmental think tank.Developed countries, including in Europe, argue that more countries need to contribute funding for efforts to tackle climate change, including wealthier developing nations such as China and oil-rich Middle Eastern states order to reach an ambitious target.Developing countries such as G20 host Brazil have pushed back on calls for obligatory contributions from anyone but developed countries, the main culprits for causing climate change.G20 nations are seen as vital to shaping the response to global warming, as they control 85% of the world economy and are also responsible for more than three-quarters of climate-warming emissions.The G20 also committed to agreeing on a legally binding treaty to limit plastic pollution by the end of 2024, with talks resuming next week to hammer out a deal two years in the making."</t>
-  </si>
-  <si>
-    <t>CC_009</t>
-  </si>
-  <si>
-    <t>The Social Democrats has said that the nitrates derogation “cannot continue and must be phased out in a controlled manner” in its General Election 2024 manifesto, which was released today (Tuesday, November 19).Last week, Social Democrats TD Jennifer Whitmore said that the party would not promise it would work to retain the derogation, and that “all the indications from Europe is that the derogation will not be available to us”.However, the Social Democrats’ manifesto has gone a step further, with the party stating that the derogation must come to an end.The party’s position on the derogation is outlined under the heading of ‘A Fair Transition for Farmers’.This also includes a commitment to incentivise a herd reduction, with the party calling for policymakers to “find a way for farmers to act in-line with national policy goals while maintaining living standards”.According to the party, some sectors “will need to be scaled back in line with our climate targets”, and that it would work to diversify the incomes of farmers in those sectors, including into energy production.However, the party also envisages farmers leaving the sector, saying that funding should be ringfenced to provide them with support and funding for education and training in other areas with employment prospects.The Social Democrats wants to design a framework of incentives to use land for tillage rather than dairy, as part of a move towards greater uptake of tillage farming.The Social Democrats said that a “key part” of agriculture policy must be to reach the sector’s emissions reduction targets while “ensuring that farmers are adequately assisted to implement, and compensated for, the changes they must make”.The party said that, if in government, it will engage with stakeholders, including farmers and their communities, to “map out a coherent transition plan” so farmers do not “disproportionately bear the brunt the transition”.As part of that, the party said it would create a €1.5 billion “Fair Transition Fund”. This would provide for a debt forgiveness scheme and a grant funding scheme that would “allow indebted farms to move away from current models of farming without undue financial loss”.The Social Democrats, if in government, would also aim to reconfigure money flowing into the sector to make farms more sustainable and to incentivise good environmental practices.On the Common Agricultural Policy (CAP), the Social Democrats intends to use the CAP Strategic Plan to “select instruments and measures that best support the delivery of all policy goals, not just in agriculture”.The party has also called for a simpler CAP that “ensures more farm payments are targeted towards low-income farmers”.The party also wants to work to increase the environmental ambition of CAP, so that farmers would only have access to payments if they “comply with a set of basic environmental norms”.Separately, the Social Democrats also wants to reform the Agri-Food Regulator as an Independent National Food Regulator (INFR), which would be tasked with enforcing EU-wide rules on unfair trading practices (UTPs).The party said it would also design a framework to restrict below-cost procurement by larger retailers, wholesalers and food processors.On live exports, the party said it would begin the process of phasing this out, and in the meantime would ban live exports to countries with lower animal welfare standards."</t>
   </si>
 </sst>
 </file>
@@ -131,8 +119,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -446,88 +437,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DACFBF2-2B92-4C4C-AF1C-30CB98805795}">
-  <dimension ref="A1:B10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF71E5E-60BE-7A42-B688-C3F104C40787}">
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>